<commit_message>
update UserAssets and translations
</commit_message>
<xml_diff>
--- a/Southwind.Terminal/InstanceTranslations/Category.de.View.xlsx
+++ b/Southwind.Terminal/InstanceTranslations/Category.de.View.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x15">
-  <x:fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<x:workbook xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <x:fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27328"/>
   <x:workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\IntTec\Extensions\Signum.Engine.Extensions\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\code\VdS\Framework\Extensions\Signum.Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{477A6F4C-E641-45FD-B2F8-0ADB0BDF64AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <x:bookViews>
-    <x:workbookView xWindow="1995" yWindow="60" windowWidth="20115" windowHeight="10515"/>
+    <x:workbookView xWindow="28680" yWindow="-2625" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </x:sheets>
-  <x:calcPr calcId="125725"/>
+  <x:calcPr calcId="152511"/>
 </x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>HeaderCell</t>
   </si>
@@ -46,20 +47,38 @@
   </si>
   <si>
     <t>Percentage</t>
+  </si>
+  <si>
+    <t>Hour</t>
+  </si>
+  <si>
+    <t>Boolean</t>
+  </si>
+  <si>
+    <t>Multiline</t>
+  </si>
+  <si>
+    <t>Apple
+Orange</t>
+  </si>
+  <si>
+    <t>Hola</t>
+  </si>
+  <si>
+    <t>Hallo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="7">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="6">
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy\ hh:mm:ss"/>
     <numFmt numFmtId="165" formatCode="_-[$£-809]* #,##0.00_-;\-[$£-809]* #,##0.00_-;_-[$£-809]* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="167" formatCode="[$¥-804]#,##0.00"/>
-    <numFmt numFmtId="168" formatCode="[$£-809]#,##0.00"/>
-    <numFmt numFmtId="169" formatCode="[$$-409]#,##0.00"/>
-    <numFmt numFmtId="170" formatCode="0&quot; km&quot;"/>
+    <numFmt numFmtId="167" formatCode="[$£-809]#,##0.00"/>
+    <numFmt numFmtId="168" formatCode="0&quot; km&quot;"/>
+    <numFmt numFmtId="169" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -126,29 +145,30 @@
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="4" applyFont="1"/>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="4" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
-    <cellStyle name="Prozent" xfId="4" builtinId="5"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
-    <cellStyle name="Überschrift" xfId="2" builtinId="15"/>
-    <cellStyle name="Überschrift 2" xfId="1" builtinId="17"/>
-    <cellStyle name="Währung" xfId="3" builtinId="4"/>
+    <cellStyle name="Currency" xfId="3" builtinId="4"/>
+    <cellStyle name="Heading 2" xfId="1" builtinId="17"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="4" builtinId="5"/>
+    <cellStyle name="Title" xfId="2" builtinId="15"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -164,9 +184,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -204,9 +224,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -241,7 +261,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -276,7 +296,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -458,460 +478,460 @@
     <x:col min="5" max="5" width="50" bestFit="1" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row>
-      <x:c s="1" t="inlineStr">
+    <x:row r="1">
+      <x:c r="A1" s="1" t="inlineStr">
         <x:is>
           <x:t>Instance</x:t>
         </x:is>
       </x:c>
-      <x:c s="1" t="inlineStr">
+      <x:c r="B1" s="1" t="inlineStr">
         <x:is>
           <x:t>Path</x:t>
         </x:is>
       </x:c>
-      <x:c s="1" t="inlineStr">
+      <x:c r="C1" s="1" t="inlineStr">
         <x:is>
           <x:t>RowId</x:t>
         </x:is>
       </x:c>
-      <x:c s="1" t="inlineStr">
+      <x:c r="D1" s="1" t="inlineStr">
         <x:is>
           <x:t>Original</x:t>
         </x:is>
       </x:c>
-      <x:c s="1" t="inlineStr">
+      <x:c r="E1" s="1" t="inlineStr">
         <x:is>
           <x:t>Translated</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t>Category;1</x:t>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+    <x:row r="2">
+      <x:c r="A2" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Category;1;Beverages</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B2" s="6" t="inlineStr">
         <x:is>
           <x:t>CategoryName</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="C2" s="6" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D2" s="6" t="inlineStr">
         <x:is>
           <x:t>Beverages</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="E2" s="6" t="inlineStr">
         <x:is>
           <x:t>Getränke</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t>Category;1</x:t>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+    <x:row r="3">
+      <x:c r="A3" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Category;1;Beverages</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B3" s="6" t="inlineStr">
         <x:is>
           <x:t>Description</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="C3" s="6" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D3" s="6" t="inlineStr">
         <x:is>
           <x:t>Soft drinks, coffees, teas, beers, and ales</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="E3" s="6" t="inlineStr">
         <x:is>
           <x:t>Softdrinks, Kaffee, Tees, Biere und Ales</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t>Category;2</x:t>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+    <x:row r="4">
+      <x:c r="A4" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Category;2;Condiments</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B4" s="6" t="inlineStr">
         <x:is>
           <x:t>CategoryName</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="C4" s="6" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D4" s="6" t="inlineStr">
         <x:is>
           <x:t>Condiments</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="E4" s="6" t="inlineStr">
         <x:is>
           <x:t>Gewürze</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t>Category;2</x:t>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+    <x:row r="5">
+      <x:c r="A5" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Category;2;Condiments</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B5" s="6" t="inlineStr">
         <x:is>
           <x:t>Description</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="C5" s="6" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D5" s="6" t="inlineStr">
         <x:is>
           <x:t>Sweet and savory sauces, relishes, spreads, and seasonings</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="E5" s="6" t="inlineStr">
         <x:is>
           <x:t>Süße und herzhafte Saucen, Relishes, Aufstriche und Gewürze</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t>Category;3</x:t>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+    <x:row r="6">
+      <x:c r="A6" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Category;3;Confections</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B6" s="6" t="inlineStr">
         <x:is>
           <x:t>CategoryName</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="C6" s="6" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D6" s="6" t="inlineStr">
         <x:is>
           <x:t>Confections</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="E6" s="6" t="inlineStr">
         <x:is>
           <x:t>Süßigkeiten</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t>Category;3</x:t>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+    <x:row r="7">
+      <x:c r="A7" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Category;3;Confections</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B7" s="6" t="inlineStr">
         <x:is>
           <x:t>Description</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="C7" s="6" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D7" s="6" t="inlineStr">
         <x:is>
           <x:t>Desserts, candies, and sweet breads</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="E7" s="6" t="inlineStr">
         <x:is>
           <x:t>Desserts, Süßigkeiten und süßebrote</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t>Category;4</x:t>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+    <x:row r="8">
+      <x:c r="A8" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Category;4;Dairy Products</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B8" s="6" t="inlineStr">
         <x:is>
           <x:t>CategoryName</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="C8" s="6" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D8" s="6" t="inlineStr">
         <x:is>
           <x:t>Dairy Products</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="E8" s="6" t="inlineStr">
         <x:is>
           <x:t>Milchprodukte</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t>Category;4</x:t>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+    <x:row r="9">
+      <x:c r="A9" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Category;4;Dairy Products</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B9" s="6" t="inlineStr">
         <x:is>
           <x:t>Description</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="C9" s="6" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D9" s="6" t="inlineStr">
         <x:is>
           <x:t>Cheeses</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="E9" s="6" t="inlineStr">
         <x:is>
           <x:t>Käse</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t>Category;5</x:t>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+    <x:row r="10">
+      <x:c r="A10" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Category;5;Grains/Cereals</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B10" s="6" t="inlineStr">
         <x:is>
           <x:t>CategoryName</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="C10" s="6" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D10" s="6" t="inlineStr">
         <x:is>
           <x:t>Grains/Cereals</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="E10" s="6" t="inlineStr">
         <x:is>
           <x:t>Körner/Getreide</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t>Category;5</x:t>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+    <x:row r="11">
+      <x:c r="A11" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Category;5;Grains/Cereals</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B11" s="6" t="inlineStr">
         <x:is>
           <x:t>Description</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="C11" s="6" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D11" s="6" t="inlineStr">
         <x:is>
           <x:t>Breads, crackers, pasta, and cereal</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="E11" s="6" t="inlineStr">
         <x:is>
           <x:t>Brote, Cracker, Nudeln und Müsli</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t>Category;6</x:t>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+    <x:row r="12">
+      <x:c r="A12" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Category;6;Meat/Poultry</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B12" s="6" t="inlineStr">
         <x:is>
           <x:t>CategoryName</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="C12" s="6" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D12" s="6" t="inlineStr">
         <x:is>
           <x:t>Meat/Poultry</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="E12" s="6" t="inlineStr">
         <x:is>
           <x:t>Fleisch/Geflügel</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t>Category;6</x:t>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+    <x:row r="13">
+      <x:c r="A13" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Category;6;Meat/Poultry</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B13" s="6" t="inlineStr">
         <x:is>
           <x:t>Description</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="C13" s="6" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D13" s="6" t="inlineStr">
         <x:is>
           <x:t>Prepared meats</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="E13" s="6" t="inlineStr">
         <x:is>
           <x:t>Zubereitetes Fleisch</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t>Category;7</x:t>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+    <x:row r="14">
+      <x:c r="A14" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Category;7;Produce</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B14" s="6" t="inlineStr">
         <x:is>
           <x:t>CategoryName</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="C14" s="6" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D14" s="6" t="inlineStr">
         <x:is>
           <x:t>Produce</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="E14" s="6" t="inlineStr">
         <x:is>
           <x:t>Frisches Obst und Gemüse</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t>Category;7</x:t>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+    <x:row r="15">
+      <x:c r="A15" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Category;7;Produce</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B15" s="6" t="inlineStr">
         <x:is>
           <x:t>Description</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="C15" s="6" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D15" s="6" t="inlineStr">
         <x:is>
           <x:t>Dried fruit and bean curd</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="E15" s="6" t="inlineStr">
         <x:is>
           <x:t>Getrocknete Früchte und Bohnenquark</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t>Category;8</x:t>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+    <x:row r="16">
+      <x:c r="A16" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Category;8;Seafood</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B16" s="6" t="inlineStr">
         <x:is>
           <x:t>CategoryName</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="C16" s="6" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D16" s="6" t="inlineStr">
         <x:is>
           <x:t>Seafood</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="E16" s="6" t="inlineStr">
         <x:is>
           <x:t>Meeresfrüchte</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t>Category;8</x:t>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+    <x:row r="17">
+      <x:c r="A17" s="6" t="inlineStr">
+        <x:is>
+          <x:t>Category;8;Seafood</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B17" s="6" t="inlineStr">
         <x:is>
           <x:t>Description</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
-        <x:is>
-          <x:t/>
-        </x:is>
-      </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="C17" s="6" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D17" s="6" t="inlineStr">
         <x:is>
           <x:t>Seaweed and fish</x:t>
         </x:is>
       </x:c>
-      <x:c s="6" t="inlineStr">
+      <x:c r="E17" s="6" t="inlineStr">
         <x:is>
           <x:t>Algen und Fische</x:t>
         </x:is>

</xml_diff>